<commit_message>
Synced Excel tables from Markdown
</commit_message>
<xml_diff>
--- a/tables/table_Campylobacter.xlsx
+++ b/tables/table_Campylobacter.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,21 +413,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>年度</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>報告機関 ／ 報告プロジェクト</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>整理状況</t>
         </is>
@@ -516,29 +504,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>**国立医薬品食品衛生研究所** &lt;br&gt; 厚生労働科学研究費（食品の安全確保推進研究事業）&lt;br&gt;「畜産食品の生物学的ハザードとそのリスクを低減するための研究」&lt;br&gt;分担研究報告書[「鶏肉食品におけるカンピロバクター等の定量的汚染実態に関する研究」](https://mhlw-grants.niph.go.jp/system/files/report_pdf/R3%E6%9C%9D%E5%80%89%E5%88%86%E6%8B%85%E7%A0%94%E7%A9%B6%E5%A0%B1%E5%91%8A%E6%9B%B8.doc__0.pdf)</t>
+          <t>**国立医薬品食品衛生研究所** &lt;br&gt; [食鳥処理場における鶏肉のカンピロバクター汚染の定量調査](https://agriknowledge.affrc.go.jp/RN/2010942163.pdf)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>未登録</t>
+          <t>済</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019-2021</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>**国立医薬品食品衛生研究所** &lt;br&gt; [食鳥処理場における鶏肉のカンピロバクター汚染の定量調査](https://agriknowledge.affrc.go.jp/RN/2010942163.pdf)</t>
+          <t>**国立医薬品食品衛生研究所** &lt;br&gt; 厚生労働科学研究費（食品の安全確保推進研究事業）&lt;br&gt;「畜産食品の生物学的ハザードとそのリスクを低減するための研究」&lt;br&gt;分担研究報告書[「鶏肉食品におけるカンピロバクター等の定量的汚染実態に関する研究」](https://mhlw-grants.niph.go.jp/system/files/report_pdf/R3%E6%9C%9D%E5%80%89%E5%88%86%E6%8B%85%E7%A0%94%E7%A9%B6%E5%A0%B1%E5%91%8A%E6%9B%B8.doc__0.pdf) &lt;br&gt;（参考: [令和1年度報告書](https://mhlw-grants.niph.go.jp/system/files/2019/193031/201924021A_upload/201924021A0004.pdf)、[令和2年度報告書](https://mhlw-grants.niph.go.jp/system/files/report_pdf/202024029A-buntan1.pdf)、[令和3年度報告書](https://mhlw-grants.niph.go.jp/system/files/report_pdf/R3%E6%9C%9D%E5%80%89%E5%88%86%E6%8B%85%E7%A0%94%E7%A9%B6%E5%A0%B1%E5%91%8A%E6%9B%B8.doc__0.pdf) ）</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -550,12 +538,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2018, 2020</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>**国立医薬品食品衛生研究所** &lt;br&gt; 厚生労働科学研究費（食品の安全確保推進研究事業）&lt;br&gt;「畜産食品の生物学的ハザードとそのリスクを低減するための研究」&lt;br&gt;分担研究報告書[「鶏肉食品におけるカンピロバクター等の定量的汚染実態に関する研究」](https://mhlw-grants.niph.go.jp/system/files/report_pdf/202024029A-buntan1.pdf)</t>
+          <t>**国立医薬品食品衛生研究所** &lt;br&gt; [2食鳥処理場におけるブロイラー群および胸肉のカンピロバクターおよびサルモネラ汚染状況と薬剤耐性](https://agriknowledge.affrc.go.jp/RN/2010937017.pdf)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -567,12 +555,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2016-2017</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>**国立医薬品食品衛生研究所** &lt;br&gt; 厚生労働科学研究費（食品の安全確保推進研究事業）&lt;br&gt;「畜産食品の生物学的ハザードとそのリスクを低減するための研究」&lt;br&gt;分担研究報告書[「鶏肉食品におけるカンピロバクター等の定量的汚染実態に関する研究」](https://mhlw-grants.niph.go.jp/system/files/2019/193031/201924021A_upload/201924021A0004.pdf)</t>
+          <t>**新潟県長岡食肉衛生検査センター** &lt;br&gt; [新潟県における市販鶏肉のカンピロバクター汚染調査](https://www.jstage.jst.go.jp/article/jvma/71/3/71_149/_pdf)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -584,12 +572,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2018, 2020</t>
+          <t>2014-2015</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>**国立医薬品食品衛生研究所** &lt;br&gt; [2食鳥処理場におけるブロイラー群および胸肉のカンピロバクターおよびサルモネラ汚染状況と薬剤耐性](https://agriknowledge.affrc.go.jp/RN/2010937017.pdf)</t>
+          <t>**一般社団法人岩手県獣医師会食烏検査センター** &lt;br&gt; [特殊飼料を給与したブロイラーでみられたカンピロバクター低汚染鶏群と偶発的区分処理の潜在的効果](https://agriknowledge.affrc.go.jp/RN/2010902975.pdf)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -601,12 +589,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>**新潟県長岡食肉衛生検査センター** &lt;br&gt; [新潟県における市販鶏肉のカンピロバクター汚染調査](https://www.jstage.jst.go.jp/article/jvma/71/3/71_149/_pdf)</t>
+          <t>**国立医薬品食品衛生研究所** &lt;br&gt; 厚生労働科学研究費（食品の安全確保推進研究事業）&lt;br&gt; [と畜・食鳥検査における疾病診断の標準化とカンピロバクター等の制御に関する研究](https://mhlw-grants.niph.go.jp/project/24503)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -618,12 +606,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2014-2015</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>**一般社団法人岩手県獣医師会食烏検査センター** &lt;br&gt; [特殊飼料を給与したブロイラーでみられたカンピロバクター低汚染鶏群と偶発的区分処理の潜在的効果](https://agriknowledge.affrc.go.jp/RN/2010902975.pdf)</t>
+          <t>**農林水産省** &lt;br&gt; [ブロイラー鶏群から製造された中抜きと体のカンピロバクター濃度調査](https://www.maff.go.jp/j/syouan/seisaku/kekka/keiniku_cam_13.html)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -635,12 +623,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>**国立医薬品食品衛生研究所** &lt;br&gt; 厚生労働科学研究費（食品の安全確保推進研究事業）&lt;br&gt; [と畜・食鳥検査における疾病診断の標準化とカンピロバクター等の制御に関する研究](https://mhlw-grants.niph.go.jp/project/24503)</t>
+          <t>**岐阜県食肉衛生検査所** &lt;br&gt; [牛胆嚢内胆汁のカンピロバクター汚染と胆汁の生化学的性状](https://warp.ndl.go.jp/info:ndljp/pid/11533510/www.pref.gifu.lg.jp/kurashi/shoku/shokuhin/22513/gakkai-tou-happyou.data/24-13.pdf)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -652,80 +640,80 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>**農林水産省** &lt;br&gt; [ブロイラー鶏群から製造された中抜きと体のカンピロバクター濃度調査](https://www.maff.go.jp/j/syouan/seisaku/kekka/keiniku_cam_13.html)</t>
+          <t>**公益財団法人鹿児島市獣医公衆衛生協会** &lt;br&gt; [食鳥処理工程におけるカンピロバクター等微生物汚染防止低減への取り組みについて](https://warp.ndl.go.jp/info:ndljp/pid/12996857/www.jyuieisei-kgo.jp/topics/sozai/researchextract01_2011.pdf)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>済</t>
+          <t>未登録</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>**岐阜県食肉衛生検査所** &lt;br&gt; [牛胆嚢内胆汁のカンピロバクター汚染と胆汁の生化学的性状](https://warp.ndl.go.jp/info:ndljp/pid/11533510/www.pref.gifu.lg.jp/kurashi/shoku/shokuhin/22513/gakkai-tou-happyou.data/24-13.pdf)</t>
+          <t>**農林水産省** &lt;br&gt; [ブロイラー鶏群から製造された中抜きと体及び鶏肉のカンピロバクター濃度調査](https://warp.ndl.go.jp/info:ndljp/pid/9534028/www.maff.go.jp/j/syouan/seisaku/kekka/keiniku_cam_07.html) &lt;br&gt; - 関連論文の[リンク](https://onlinelibrary.wiley.com/doi/10.1111/j.1863-2378.2012.01509.x)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>未登録</t>
+          <t>済</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2004-2011</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>**公益財団法人鹿児島市獣医公衆衛生協会** &lt;br&gt; [食鳥処理工程におけるカンピロバクター等微生物汚染防止低減への取り組みについて](https://warp.ndl.go.jp/info:ndljp/pid/12996857/www.jyuieisei-kgo.jp/topics/sozai/researchextract01_2011.pdf)</t>
+          <t>**埼玉県衛生研究所** &lt;br&gt; [市販鶏肉のカンピロバクター及びサルモネラ汚染状況と分離株の薬剤感受性](https://jvma-vet.jp/mag/06706/d2.pdf) &lt;br&gt;（日本獣医師会雑誌, 67巻, 442~448, 2014）</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>未登録</t>
+          <t>済</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>**農林水産省** &lt;br&gt; [ブロイラー鶏群から製造された中抜きと体及び鶏肉のカンピロバクター濃度調査](https://warp.ndl.go.jp/info:ndljp/pid/9534028/www.maff.go.jp/j/syouan/seisaku/kekka/keiniku_cam_07.html) &lt;br&gt; - 関連論文の[リンク](https://onlinelibrary.wiley.com/doi/10.1111/j.1863-2378.2012.01509.x)</t>
+          <t>**宮城県保健環境センター** &lt;br&gt; [市販食肉等からのカンピロバクター検出と低温保存での菌消長](https://www.pref.miyagi.jp/documents/1979/209066.pdf)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>済</t>
+          <t>未登録</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2004-2011</t>
+          <t>2001</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>**埼玉県衛生研究所** &lt;br&gt; [市販鶏肉のカンピロバクター及びサルモネラ汚染状況と分離株の薬剤感受性](https://jvma-vet.jp/mag/06706/d2.pdf) &lt;br&gt;（日本獣医師会雑誌, 67巻, 442~448, 2014）</t>
+          <t>**埼玉県衛生研究所** &lt;br&gt; [MPN法および直接平板塗抹法による市販鶏レバーのカンピロバクターの定量検査](https://www.jstage.jst.go.jp/article/jvma1951/55/7/55_7_447/_pdf/-char/en) &lt;br&gt;（日本獣医師会雑誌, 55巻, 447~449, 2002）</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -737,12 +725,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>2000-2001</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>**宮城県保健環境センター** &lt;br&gt; [市販食肉等からのカンピロバクター検出と低温保存での菌消長](https://www.pref.miyagi.jp/documents/1979/209066.pdf)</t>
+          <t>**岩手大学** &lt;br&gt; 厚生労働科学研究費（特別研究事業） &lt;br&gt; [鶏肉に起因するカンピロバクター食中毒の予防対策に関する調査研究](https://warp.ndl.go.jp/collections/content/info:ndljp/pid/13046218/mhlw-grants.niph.go.jp/project/3941)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -754,66 +742,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>**埼玉県衛生研究所** &lt;br&gt; [MPN法および直接平板塗抹法による市販鶏レバーのカンピロバクターの定量検査](https://www.jstage.jst.go.jp/article/jvma1951/55/7/55_7_447/_pdf/-char/en) &lt;br&gt;（日本獣医師会雑誌, 55巻, 447~449, 2002）</t>
+          <t>**埼玉県衛生研究所** &lt;br&gt; [市販鶏肉におけるカンピロバクターの定量検査と分離菌株の血清型](https://www.jstage.jst.go.jp/article/jvma1951/57/9/57_9_595/_pdf/-char/ja) &lt;br&gt;（日本獣医師会雑誌, 57巻, 595~598, 2004）</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>済</t>
+          <t>未登録</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2000-2001</t>
+          <t>1999-2002</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>**岩手大学** &lt;br&gt; 厚生労働科学研究費（特別研究事業） &lt;br&gt; [鶏肉に起因するカンピロバクター食中毒の予防対策に関する調査研究](https://warp.ndl.go.jp/collections/content/info:ndljp/pid/13046218/mhlw-grants.niph.go.jp/project/3941)</t>
+          <t>**埼玉県衛生研究所** &lt;br&gt; [国産および輸入鶏肉におけるカンピロバクターの汚染状況](https://agriknowledge.affrc.go.jp/RN/2010671140.pdf) &lt;br&gt;（日本獣医師会雑誌, 56巻, 103~105, 2003）&lt;br&gt; 2000年以降のデータ（国産鶏肉）のみ追加</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
-        <is>
-          <t>未登録</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>**埼玉県衛生研究所** &lt;br&gt; [市販鶏肉におけるカンピロバクターの定量検査と分離菌株の血清型](https://www.jstage.jst.go.jp/article/jvma1951/57/9/57_9_595/_pdf/-char/ja) &lt;br&gt;（日本獣医師会雑誌, 57巻, 595~598, 2004）</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>未登録</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>1999-2002</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>**埼玉県衛生研究所** &lt;br&gt; [国産および輸入鶏肉におけるカンピロバクターの汚染状況](https://agriknowledge.affrc.go.jp/RN/2010671140.pdf) &lt;br&gt;（日本獣医師会雑誌, 56巻, 103~105, 2003）&lt;br&gt; 2000年以降のデータ（国産鶏肉）のみ追加</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
         <is>
           <t>未登録</t>
         </is>

</xml_diff>